<commit_message>
feat(design): adoption de la palette medicale officielle en tokens Tailwind 4
- 9 couleurs PO mappees en tokens semantiques (globals.css, ADR-002)
- nouveaux tokens success/warning/primary-dark + mapping @theme inline
- contrastes WCAG AA verifies (blanc interdit sur success/warning)
- theme sombre par nuances derivees documentees (DESIGN_SYSTEM §1.4)
- verifie: lint 0 err., 8/8 hex servis, computed styles conformes (agent-browser)

Refs: ADR-002, DESIGN-T01, SYS-008
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASKS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T12"/>
+  <dimension ref="B2:T13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -869,108 +869,205 @@
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DESIGN-T01</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Palette médicale</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Tokens + documentation</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Implémentation des 9 couleurs du PO en tokens Tailwind 4 (globals.css) ; règles d'usage sémantique ; contrastes WCAG AA ; ADR-002</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>UX/UI + Frontend + Tech Lead</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>SYS-T01</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>src/app/globals.css · .ai/DESIGN_SYSTEM.md §1 · .ai/ADR/ADR-002</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>lint · CSS servi (grep hex) · agent-browser computed styles</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Lint 0 erreur · 8/8 hex servis · tokens calculés conformes</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>feat(design)</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED (revue interne Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>Contrastes : texte blanc interdit sur success/warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>En attente de demandes utilisateur</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Aucune feature métier demandée à ce jour ; le backlog sera alimenté par le PO (utilisateur)</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr"/>
+      <c r="S9" s="3" t="inlineStr"/>
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>Feature Lifecycle (WORKFLOWS.md) appliqué à chaque demande</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
           <t>Règles de blocage : Frontend bloqué sans contrat API validé · PROD bloquée sans audit global ≥ 60/100 · FRONTEND TERMINÉ exige a11y + perf validés.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:T8"/>
+  <autoFilter ref="B4:T9"/>
   <mergeCells count="1">
     <mergeCell ref="B2:T2"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(gouvernance): clôture BUG-001/OPS-T01 dans les registres et worklog
Refs: BUG-001, OPS-T01, SEC-ADV-001
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASKS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T13"/>
+  <dimension ref="B2:T15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -966,108 +966,302 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BUG-T01</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BUG-001 hydratation</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Fix layout</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>suppressHydrationWarning sur &lt;body&gt; (attributs injectés par l'environnement preview : bis_status, __processed_*)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>DEV Frontend + QA</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>DESIGN-T01</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>src/app/layout.tsx · .ai/BUGS.md</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>agent-browser reload (0 erreur, console propre) · lint</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Lint 0 erreur · 0 erreur page</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>BUG-001 corrigé</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>fix(ui) 13d8d92</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED (revue interne Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Cause externe confirmée (absence bis_* en headless)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>OPS-T01</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Push GitHub</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Synchronisation remote</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Push de main vers github.com/akoun-dev/mondocpro.git (token PO one-shot, non persisté) + retrait .env/db du suivi git</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>DEVOPS + COMMIT + Security</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>BUG-T01</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>remote origin · .gitignore · .env (untrack) · db/custom.db (untrack)</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>git ls-remote post-push</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Hash remote 90786c8 = local</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>chore(securite) 90786c8</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>n/a (ops)</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>SEC-ADV-001 : rotation du token conseillée (action PO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>En attente de demandes utilisateur</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Aucune feature métier demandée à ce jour ; le backlog sera alimenté par le PO (utilisateur)</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R9" s="3" t="inlineStr"/>
-      <c r="S9" s="3" t="inlineStr"/>
-      <c r="T9" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr"/>
+      <c r="S11" s="3" t="inlineStr"/>
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>Feature Lifecycle (WORKFLOWS.md) appliqué à chaque demande</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Règles de blocage : Frontend bloqué sans contrat API validé · PROD bloquée sans audit global ≥ 60/100 · FRONTEND TERMINÉ exige a11y + perf validés.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:T9"/>
+  <autoFilter ref="B4:T11"/>
   <mergeCells count="1">
     <mergeCell ref="B2:T2"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat(data): migration de la base vers supabase postgresql
- provider prisma sqlite->postgresql (ADR-003)
- connexion via pooler supavisor IPv4 session mode (host direct IPv6-only,
  region aws-1-eu-west-1 identifiee par auth reelle)
- schema User/Post synchronise ; roundtrip SELECT 1 verifie ; REST 200
- scripts db:* blindes contre l'override DATABASE_URL du shell sandbox
- secrets en .env non versionne (SEC-ADV-002 : rotation conseillee)

Refs: ADR-003, DB-T01, SYS-009
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASKS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T15"/>
+  <dimension ref="B2:T16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1160,108 +1160,205 @@
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DB-T01</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Supabase PostgreSQL</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Migration BDD</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Provider prisma sqlite→postgresql ; pooler Supavisor IPv4 (host direct IPv6-only) ; région aws-1-eu-west-1 découverte par auth réelle ; schéma User/Post synchronisé ; scripts db:* blindés ; secrets en .env non versionné</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>DEVOPS/DATA + Tech Lead + Security</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>OPS-T01</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>prisma/schema.prisma · .env · package.json · .ai/ADR/ADR-003</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Roundtrip Prisma SELECT 1 · REST /rest/v1/User · GET / post-restart</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Roundtrip OK · REST 200 [] · lint 0 erreur</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>feat(data)</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED (revue interne Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>ADR-003 · SEC-ADV-002 : rotation secrets Supabase conseillée · migrations versionnées avant PROD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>En attente de demandes utilisateur</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Aucune feature métier demandée à ce jour ; le backlog sera alimenté par le PO (utilisateur)</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R11" s="3" t="inlineStr"/>
-      <c r="S11" s="3" t="inlineStr"/>
-      <c r="T11" s="3" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr">
         <is>
           <t>Feature Lifecycle (WORKFLOWS.md) appliqué à chaque demande</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
+          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
           <t>Règles de blocage : Frontend bloqué sans contrat API validé · PROD bloquée sans audit global ≥ 60/100 · FRONTEND TERMINÉ exige a11y + perf validés.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:T11"/>
+  <autoFilter ref="B4:T12"/>
   <mergeCells count="1">
     <mergeCell ref="B2:T2"/>
   </mergeCells>

</xml_diff>

<commit_message>
chore(devops): flux de boot custom resistant au cold start (dev.sh)
- restaure .env supabase (ecrase par /start.sh a chaque boot)
- bun install + db:push + serveur, via le flux custom de la plateforme
- test_db.ts autonome (lit .env, immunise a l'export shell herite)

Refs: OPS-T02, ADR-003
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASKS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T16"/>
+  <dimension ref="B2:T17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1160,67 +1160,67 @@
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>OPS-T02</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Résilience boot</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>dev.sh custom</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>/start.sh écrase .env (file:...) à chaque cold start → flux custom .zscripts/dev.sh (restaure .env Supabase depuis .zscripts/.env.supabase non versionné, bun install, db:push, dev) + relance serveur vérifiée cross-session</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>DEVOPS/DATA</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
           <t>DB-T01</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Supabase PostgreSQL</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Migration BDD</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Provider prisma sqlite→postgresql ; pooler Supavisor IPv4 (host direct IPv6-only) ; région aws-1-eu-west-1 découverte par auth réelle ; schéma User/Post synchronisé ; scripts db:* blindés ; secrets en .env non versionné</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>DEVOPS/DATA + Tech Lead + Security</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>TERMINÉ</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>OPS-T01</t>
-        </is>
-      </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>prisma/schema.prisma · .env · package.json · .ai/ADR/ADR-003</t>
+          <t>.zscripts/dev.sh · .zscripts/.env.supabase (non versionné)</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Roundtrip Prisma SELECT 1 · REST /rest/v1/User · GET / post-restart</t>
+          <t>curl 200 cross-session · Caddy :81 200 · test_db SELECT 1</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Roundtrip OK · REST 200 [] · lint 0 erreur</t>
+          <t>200 · 200 · OK</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>feat(data)</t>
+          <t>chore(devops)</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>APPROVED (revue interne Tech Lead)</t>
+          <t>n/a (ops)</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1250,115 +1250,212 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>ADR-003 · SEC-ADV-002 : rotation secrets Supabase conseillée · migrations versionnées avant PROD</t>
+          <t>Secrets protégés (.gitignore .env*) ; flux boot validé</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>DB-T01</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PostgreSQL</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Migration BDD</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Provider prisma sqlite→postgresql ; pooler Supavisor IPv4 (host direct IPv6-only) ; région aws-1-eu-west-1 découverte par auth réelle ; schéma User/Post synchronisé ; scripts db:* blindés ; secrets en .env non versionné</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>DEVOPS/DATA + Tech Lead + Security</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>OPS-T01</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>prisma/schema.prisma · .env · package.json · .ai/ADR/ADR-003</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Roundtrip Prisma SELECT 1 · REST /rest/v1/User · GET / post-restart</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Roundtrip OK · REST 200 [] · lint 0 erreur</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>feat(data)</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED (revue interne Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>ADR-003 · SEC-ADV-002 : rotation secrets Supabase conseillée · migrations versionnées avant PROD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>En attente de demandes utilisateur</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Aucune feature métier demandée à ce jour ; le backlog sera alimenté par le PO (utilisateur)</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="P13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="R12" s="4" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr">
+      <c r="R13" s="3" t="inlineStr"/>
+      <c r="S13" s="3" t="inlineStr"/>
+      <c r="T13" s="3" t="inlineStr">
         <is>
           <t>Feature Lifecycle (WORKFLOWS.md) appliqué à chaque demande</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
           <t>Règles de blocage : Frontend bloqué sans contrat API validé · PROD bloquée sans audit global ≥ 60/100 · FRONTEND TERMINÉ exige a11y + perf validés.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:T12"/>
+  <autoFilter ref="B4:T13"/>
   <mergeCells count="1">
     <mergeCell ref="B2:T2"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(gouvernance): registre OPS-T03 et journal des commits complete
- TASKS.md/xlsx : OPS-T03 (xlsx validate 0 issue)
- CHANGELOG + PROJECT_CONTEXT : guide configuration locale
- COMMIT_LOG : comblement des entrees manquantes (7657ee2, ace3161, c6b1d34, d1370c3) + audit auto-commit 0badaee
- worklog Task 6
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASKS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T17"/>
+  <dimension ref="B2:T18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1354,108 +1354,205 @@
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
+          <t>OPS-T03</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Config locale reproductible</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Modèle .env.example</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>.env.example versionné (placeholders uniquement, zéro secret — scan avant commit) + exception .gitignore !.env.example ; instructions pas-à-pas de configuration locale Supabase (cp .env.example .env → db:push → dev)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>DEVOPS + Doc + Security</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>DB-T01</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>.env.example · .gitignore</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Scan anti-secret · git check-ignore (.env/.env.supabase toujours ignorés) · lint</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>0 secret · tracking OK · lint 0 erreur</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>chore(env)</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>n/a (ops)</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>SEC-ADV-002 reste ouverte (rotation secrets = action PO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>En attente de demandes utilisateur</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Aucune feature métier demandée à ce jour ; le backlog sera alimenté par le PO (utilisateur)</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="R13" s="3" t="inlineStr"/>
-      <c r="S13" s="3" t="inlineStr"/>
-      <c r="T13" s="3" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr">
         <is>
           <t>Feature Lifecycle (WORKFLOWS.md) appliqué à chaque demande</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
           <t>Règles de blocage : Frontend bloqué sans contrat API validé · PROD bloquée sans audit global ≥ 60/100 · FRONTEND TERMINÉ exige a11y + perf validés.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:T13"/>
+  <autoFilter ref="B4:T14"/>
   <mergeCells count="1">
     <mergeCell ref="B2:T2"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs(gouvernance): registres feature auth (spec, adr, contrats, tasks, tests)
- SPEC-AUTH.md (phase 0-1) + ADR-004 + 4 contrats API valides
- TASKS.md/xlsx : AUTH-T01..04 terminees (validate 0 issue)
- TEST_PLAN : 7 scenarios PASS · REQUIREMENTS SYS-010 · TEAM_STATUS
- worklog Task 7 (orchestrateur) + section 7-d (subagent frontend)

Refs: AUTH-T01..T04, SYS-010
</commit_message>
<xml_diff>
--- a/.ai/TASKS.xlsx
+++ b/.ai/TASKS.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TASKS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TASKS'!$B$4:$T$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:T18"/>
+  <dimension ref="B2:T22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1451,108 +1451,496 @@
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>AUTH-T01</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>FEATURE-AUTH</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Schéma Prisma auth</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>User métier (phone unique, passwordHash, role, zone) + Session (tokenHash, expiresAt) ; enums Role/Zone ; suppression scaffold Post ; db push Supabase + seed Dr Kadjane (ADMIN_INITIAL_PASSWORD)</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>DEVOPS/DATA</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>OPS-T03</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>prisma/schema.prisma · .zscripts/seed_admin.ts · .env.example</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>db push · seed exécuté · login admin</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Push 10.65s OK · seed Dr Kadjane OK · login admin 200</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>feat(data)</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED (revue Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>ADR-004 · bcrypt 10 rounds · token session hashé SHA-256 en DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>AUTH-T02</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>FEATURE-AUTH</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Service + API auth</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>src/lib/auth.ts (bcrypt 10, sessions SHA-256, cookie httpOnly 30j) + routes /api/auth/register·login·me·logout (zod, enveloppe standard)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>DEV Backend + Security</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>AUTH-T01</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>src/lib/auth.ts · src/app/api/auth/**</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>curl 4 routes (9 cas : 201/409/400/200/401 + cookie HttpOnly)</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>9/9 conformes aux contrats</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>feat(api)</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED (revue Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Anti-énumération (hash factice) · fix dev.sh : export DATABASE_URL depuis .env</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-T03</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>FEATURE-AUTH</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Écran auth + espace connecté</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>layout.tsx (fr, meta MondocPro, icône PO) + page.tsx orchestration (checking/auth/dashboard) + composants auth/ + store zustand + hook useAuth ; palette médicale, mobile-first, a11y AA, footer sticky</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>DEV Frontend + UX/UI</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-T02</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>src/app/layout.tsx · src/app/page.tsx · src/components/auth/** · src/stores/** · src/hooks/**</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Browser E2E 10 étapes + lint + tsc</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>10/10 PASS · lint 0 err. · tsc 0 err. · 0 erreur console</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>feat(ui)</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED (revue Tech Lead)</t>
+        </is>
+      </c>
+      <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>Composants vides PO (admin/nurses/users) intacts · QA indépendante confirmée (mobile 375px, footer, touch ≥44px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>AUTH-T04</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>FEATURE-AUTH</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Vérification E2E</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Plan TEST_PLAN appliqué : parcours 3 rôles, guards, sécurité (hash, cookies, erreurs génériques), lint, dev.log</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>QA + Tech Lead</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>TERMINÉ</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>AUTH-T03</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>.ai/TEST_PLAN.md · agent-browser</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>7 scénarios consignés au journal des tests</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>7/7 PASS (journal TEST_PLAN)</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED (QA)</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>Détails : .ai/TEST_PLAN.md — section FEATURE-AUTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>En attente de demandes utilisateur</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Aucune feature métier demandée à ce jour ; le backlog sera alimenté par le PO (utilisateur)</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr"/>
-      <c r="S14" s="4" t="inlineStr"/>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr">
         <is>
           <t>Feature Lifecycle (WORKFLOWS.md) appliqué à chaque demande</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="5" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Statuts : À FAIRE → EN COURS → EN REVUE → TEST QA → TERMINÉ (ou BLOQUÉ). Intégrité : tout statut avancé exige une preuve (commit, revue, test, audit).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Règles de blocage : Frontend bloqué sans contrat API validé · PROD bloquée sans audit global ≥ 60/100 · FRONTEND TERMINÉ exige a11y + perf validés.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:T14"/>
+  <autoFilter ref="B4:T18"/>
   <mergeCells count="1">
     <mergeCell ref="B2:T2"/>
   </mergeCells>

</xml_diff>